<commit_message>
SSHv2.1 - Servis durumu veri akisi fix, normalize_status, grid sync, template esnek eslestirme, DB normalizasyon
</commit_message>
<xml_diff>
--- a/data/kayseri/Veriler.xlsx
+++ b/data/kayseri/Veriler.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fatiherkin\Desktop\bozankaya_ssh_takip\data\kayseri\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86824D87-6D12-47F8-B7C5-D60A266137CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B29BE82-7171-4B3E-A58F-70E58C630537}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="217">
   <si>
     <t>Traction_Converter</t>
   </si>
@@ -679,6 +679,12 @@
   </si>
   <si>
     <t>ZİL</t>
+  </si>
+  <si>
+    <t>Sürücü Kapısı</t>
+  </si>
+  <si>
+    <t>Sağ Kolçak</t>
   </si>
 </sst>
 </file>
@@ -1671,7 +1677,9 @@
       <c r="AM4" s="11"/>
       <c r="AN4" s="10"/>
       <c r="AO4" s="10"/>
-      <c r="AP4" s="10"/>
+      <c r="AP4" s="10" t="s">
+        <v>215</v>
+      </c>
     </row>
     <row r="5" spans="1:42" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
@@ -1749,7 +1757,9 @@
       <c r="AM5" s="11"/>
       <c r="AN5" s="10"/>
       <c r="AO5" s="10"/>
-      <c r="AP5" s="10"/>
+      <c r="AP5" s="10" t="s">
+        <v>216</v>
+      </c>
     </row>
     <row r="6" spans="1:42" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">

</xml_diff>